<commit_message>
feat: refresh analysis UI and workflows
</commit_message>
<xml_diff>
--- a/docs/acyl_chain_rule_table.xlsx
+++ b/docs/acyl_chain_rule_table.xlsx
@@ -230,7 +230,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -317,7 +317,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -404,7 +404,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses. Extract trailing 'FA xx:y' notation outside parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses. Extract trailing 'FA xx:y' notation outside parentheses.</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -2579,7 +2579,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -4145,7 +4145,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -4580,7 +4580,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -4841,7 +4841,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -4928,7 +4928,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5015,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -5450,7 +5450,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -5537,7 +5537,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -5624,7 +5624,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -5798,7 +5798,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -5885,7 +5885,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5972,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -6059,7 +6059,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -6494,7 +6494,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -6755,7 +6755,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -7190,7 +7190,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Extract FA-style chains from final parentheses. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Extract FA-style chains from final parentheses. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Extract FA-style chains from final parentheses. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Extract FA-style chains from final parentheses. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -7947,7 +7947,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses. Extract trailing 'FA xx:y' notation outside parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses. Extract trailing 'FA xx:y' notation outside parentheses.</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Skip sum-only notation when molecular/sn evidence is absent. Drop the first chain when two or more chain tokens are present. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -8357,7 +8357,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Extract FA-style chains from final parentheses.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Extract FA-style chains from final parentheses.</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -8603,7 +8603,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -8685,7 +8685,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -8767,7 +8767,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>
@@ -8849,7 +8849,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit. Remove zero chains such as 0:0.</t>
         </is>
       </c>
     </row>
@@ -8931,7 +8931,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Split order: '/' -&gt; '_' -&gt; whitespace -&gt; unsplit.</t>
+          <t xml:space="preserve">Split delimiters: '/' and '_' when present; otherwise whitespace -&gt; unsplit.</t>
         </is>
       </c>
     </row>

</xml_diff>